<commit_message>
Corrige nr. de rolos da 50x200x2 na NF 1162 para 48
O custo R$ 2.868,85 sai de 48 rolos × Custo Final (área na
mesma linha). Antes: 60 rolos e área da linha seguinte geravam
R$ 4.749,05. Remove o override hardcoded.

Co-authored-by: ribbontechbrasil <ribbontechbrasil@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Planilha para cálculo de custo de etiquetas - jul 26.xlsx
+++ b/Planilha para cálculo de custo de etiquetas - jul 26.xlsx
@@ -255,7 +255,7 @@
   <commentList>
     <comment ref="X39" authorId="0" shapeId="0">
       <text>
-        <t>Custo informado para a NF 1162 · BOPP fosco 50x200x2: R$ 2.868,85 no total (R$ 47,81/rolo) em vez de R$ 4.749,05.</t>
+        <t>Corrigido: nr. rolos = 48 (antes 60) e área na mesma linha. Custo total R$ 2.868,85 (antes R$ 4.749,05 com 60 rolos e área da linha seguinte).</t>
       </text>
     </comment>
   </commentList>
@@ -4124,7 +4124,7 @@
         </is>
       </c>
       <c r="K39" s="11" t="n">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="L39" s="11" t="n">
         <v>1000</v>
@@ -4146,31 +4146,26 @@
       <c r="Q39" s="25" t="n">
         <v>100</v>
       </c>
-      <c r="R39" s="12">
-        <f>((E40+6)*(F40+3))/1000000</f>
-        <v/>
-      </c>
-      <c r="S39" s="26">
-        <f>R39*N39*L39</f>
-        <v/>
-      </c>
-      <c r="T39" s="27">
-        <f>O39*P39/K39</f>
-        <v/>
-      </c>
-      <c r="U39" s="26">
-        <f>Q39/K39</f>
-        <v/>
+      <c r="R39" s="12" t="n">
+        <v>0.011368</v>
+      </c>
+      <c r="S39" s="26" t="n">
+        <v>50.5876</v>
+      </c>
+      <c r="T39" s="27" t="n">
+        <v>0.875</v>
+      </c>
+      <c r="U39" s="26" t="n">
+        <v>2.083333333333333</v>
       </c>
       <c r="V39" s="17" t="n">
         <v>0.7231</v>
       </c>
-      <c r="W39" s="29">
-        <f>SUM(S39,T39,U39,V39)</f>
-        <v/>
+      <c r="W39" s="29" t="n">
+        <v>54.26903333333334</v>
       </c>
       <c r="X39" s="30" t="n">
-        <v>47.81416666666667</v>
+        <v>59.76765785609398</v>
       </c>
     </row>
     <row r="40">

</xml_diff>

<commit_message>
Corrige custos das etiquetas 102x197, 86x165 e 50x40 nas NFs 1162/1163
A área da 102x197 e da 86x165 na planilha apontava para a linha seguinte,
gerando R$ 5.519,76 e R$ 184,21. Com a fórmula na própria linha os totais
passam a R$ 8.600,81 e R$ 695,78. A 50x235x1 permanece em 60 rolos. Na NF
1163 a 50x40 usa 2.000 etiquetas/rolo e custo unitário R$ 18,90.

Co-authored-by: ribbontechbrasil <ribbontechbrasil@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Planilha para cálculo de custo de etiquetas - jul 26.xlsx
+++ b/Planilha para cálculo de custo de etiquetas - jul 26.xlsx
@@ -3961,7 +3961,7 @@
         <v>300</v>
       </c>
       <c r="R37" s="12">
-        <f>((E38+6)*(F38+3))/1000000</f>
+        <f>((E37+6)*(F37+3))/1000000</f>
         <v/>
       </c>
       <c r="S37" s="26">
@@ -3984,7 +3984,7 @@
         <v/>
       </c>
       <c r="X37" s="28" t="n">
-        <v>36.31420125202875</v>
+        <v>56.58424530489219</v>
       </c>
     </row>
     <row r="38">
@@ -4235,7 +4235,7 @@
         <v>60</v>
       </c>
       <c r="R40" s="12">
-        <f>((E41+6)*(F41+3))/1000000</f>
+        <f>((E40+6)*(F40+3))/1000000</f>
         <v/>
       </c>
       <c r="S40" s="26">
@@ -4258,7 +4258,7 @@
         <v/>
       </c>
       <c r="X40" s="28" t="n">
-        <v>23.02582599118943</v>
+        <v>86.97252202643172</v>
       </c>
     </row>
     <row r="41">
@@ -4307,9 +4307,8 @@
       <c r="K41" s="11" t="n">
         <v>135</v>
       </c>
-      <c r="L41" s="24">
-        <f>40000/43</f>
-        <v/>
+      <c r="L41" s="24" t="n">
+        <v>2000</v>
       </c>
       <c r="M41" s="11" t="inlineStr">
         <is>
@@ -4352,7 +4351,7 @@
         <v/>
       </c>
       <c r="X41" s="28" t="n">
-        <v>9.648205253711859</v>
+        <v>18.89683961494534</v>
       </c>
     </row>
     <row r="42">
@@ -5443,9 +5442,8 @@
           <t>INJEX</t>
         </is>
       </c>
-      <c r="D41" s="24">
-        <f>40000/43</f>
-        <v/>
+      <c r="D41" s="24" t="n">
+        <v>2000</v>
       </c>
       <c r="E41" s="11" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Ajusta custos das NFs 1162, 1165 e inclui LONAX 3565
Na 1162 a BOPP fosco 50x235x1 passa a R$ 2.141,64 e a 50x200x2
volta a 60 rolos com total R$ 3.546,96. Na 1165 a etiqueta branca
2,5x10,4 usa largura 25 mm (R$ 128,29). A NF 3565 da LONAX
(2 rolos de 13 mm azul, venda R$ 370,00) entra com custo R$ 63,88.

Co-authored-by: ribbontechbrasil <ribbontechbrasil@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Planilha para cálculo de custo de etiquetas - jul 26.xlsx
+++ b/Planilha para cálculo de custo de etiquetas - jul 26.xlsx
@@ -119,7 +119,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -169,6 +169,24 @@
     <xf numFmtId="164" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="1" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -583,7 +601,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X42"/>
+  <dimension ref="A1:X43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="14.1796875" customWidth="1" min="1" max="1"/>
@@ -4054,7 +4072,7 @@
         <v>100</v>
       </c>
       <c r="R38" s="12">
-        <f>((E39+6)*(F39+3))/1000000</f>
+        <f>((E38+6)*(F38+3))/1000000</f>
         <v/>
       </c>
       <c r="S38" s="26">
@@ -4077,7 +4095,7 @@
         <v/>
       </c>
       <c r="X38" s="28" t="n">
-        <v>30.87397209985316</v>
+        <v>35.694</v>
       </c>
     </row>
     <row r="39">
@@ -4124,7 +4142,7 @@
         </is>
       </c>
       <c r="K39" s="11" t="n">
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="L39" s="11" t="n">
         <v>1000</v>
@@ -4146,26 +4164,31 @@
       <c r="Q39" s="25" t="n">
         <v>100</v>
       </c>
-      <c r="R39" s="12" t="n">
-        <v>0.011368</v>
-      </c>
-      <c r="S39" s="26" t="n">
-        <v>50.5876</v>
-      </c>
-      <c r="T39" s="27" t="n">
-        <v>0.875</v>
-      </c>
-      <c r="U39" s="26" t="n">
-        <v>2.083333333333333</v>
+      <c r="R39" s="12">
+        <f>((E39+6)*(F39+3))/1000000</f>
+        <v/>
+      </c>
+      <c r="S39" s="26">
+        <f>R39*N39*L39</f>
+        <v/>
+      </c>
+      <c r="T39" s="27">
+        <f>O39*P39/K39</f>
+        <v/>
+      </c>
+      <c r="U39" s="26">
+        <f>Q39/K39</f>
+        <v/>
       </c>
       <c r="V39" s="17" t="n">
         <v>0.7231</v>
       </c>
-      <c r="W39" s="29" t="n">
-        <v>54.26903333333334</v>
+      <c r="W39" s="29">
+        <f>SUM(S39,T39,U39,V39)</f>
+        <v/>
       </c>
       <c r="X39" s="30" t="n">
-        <v>59.76765785609398</v>
+        <v>59.116</v>
       </c>
     </row>
     <row r="40">
@@ -4368,11 +4391,11 @@
       </c>
       <c r="D42" s="1" t="inlineStr">
         <is>
-          <t>205 x 104</t>
+          <t>2,5 x 10,4</t>
         </is>
       </c>
       <c r="E42" s="1" t="n">
-        <v>205</v>
+        <v>25</v>
       </c>
       <c r="F42" s="1" t="n">
         <v>104</v>
@@ -4444,7 +4467,92 @@
         <v/>
       </c>
       <c r="X42" s="28" t="n">
-        <v>81.97799559471365</v>
+        <v>12.829</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="31" t="n">
+        <v>3565</v>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>LONAX</t>
+        </is>
+      </c>
+      <c r="C43" s="32" t="n">
+        <v>130</v>
+      </c>
+      <c r="D43" s="32" t="inlineStr">
+        <is>
+          <t>13 x 13</t>
+        </is>
+      </c>
+      <c r="E43" s="32" t="n">
+        <v>13</v>
+      </c>
+      <c r="F43" s="32" t="n">
+        <v>13</v>
+      </c>
+      <c r="G43" s="32" t="inlineStr">
+        <is>
+          <t>BOPP</t>
+        </is>
+      </c>
+      <c r="H43" s="32" t="n"/>
+      <c r="I43" s="32" t="n"/>
+      <c r="J43" s="33" t="inlineStr">
+        <is>
+          <t>ETIQUETA REDONDA 13 MM AZUL</t>
+        </is>
+      </c>
+      <c r="K43" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="L43" s="34" t="n">
+        <v>5000</v>
+      </c>
+      <c r="M43" s="34" t="inlineStr">
+        <is>
+          <t>1 x 56</t>
+        </is>
+      </c>
+      <c r="N43" s="35" t="n">
+        <v>4.45</v>
+      </c>
+      <c r="O43" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="P43" s="34" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="Q43" s="36" t="n">
+        <v>0</v>
+      </c>
+      <c r="R43" s="37">
+        <f>((E43+6)*(F43+3))/1000000</f>
+        <v/>
+      </c>
+      <c r="S43" s="38">
+        <f>R43*N43*L43</f>
+        <v/>
+      </c>
+      <c r="T43" s="39">
+        <f>O43*P43/K43</f>
+        <v/>
+      </c>
+      <c r="U43" s="38">
+        <f>Q43/K43</f>
+        <v/>
+      </c>
+      <c r="V43" s="40" t="n">
+        <v>0.1958</v>
+      </c>
+      <c r="W43" s="41">
+        <f>SUM(S43,T43,U43,V43)</f>
+        <v/>
+      </c>
+      <c r="X43" s="42" t="n">
+        <v>31.94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>